<commit_message>
Changed temp sensor, added components and created a general layout design
</commit_message>
<xml_diff>
--- a/BodyTempSensor_Calculations.xlsx
+++ b/BodyTempSensor_Calculations.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daanheetkamp/Desktop/BodyTempSensor/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EA421BB-3A52-904B-85A5-F8DC7A305473}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EC6E96C-A43A-574E-A672-C76E5C870D18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17820" xr2:uid="{40AEC5D9-C44A-0B49-91FD-EA69EB214C5D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="19">
   <si>
     <t>USB-C</t>
   </si>
@@ -137,10 +137,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -476,7 +475,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BCE080E-A5D5-DB4A-A02C-D924411D9F97}">
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.83203125" bestFit="1" customWidth="1"/>
@@ -525,15 +524,15 @@
       <c r="I2" t="s">
         <v>14</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2">
         <f>$H$1/B10</f>
         <v>60.788425883711739</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2">
         <f t="shared" ref="K2:L2" si="0">$H$1/C10</f>
         <v>32.630685897017557</v>
       </c>
-      <c r="L2" s="2">
+      <c r="L2">
         <f t="shared" si="0"/>
         <v>3149.6062992125981</v>
       </c>
@@ -612,10 +611,10 @@
         <v>1.1E-4</v>
       </c>
       <c r="E6" s="1"/>
-      <c r="I6" s="3" t="s">
+      <c r="I6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="J6" s="3"/>
+      <c r="J6" s="2"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -631,10 +630,10 @@
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="E7" s="1"/>
-      <c r="I7" s="3" t="s">
+      <c r="I7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J7" s="3"/>
+      <c r="J7" s="2"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -650,10 +649,10 @@
         <v>4.9999999999999998E-7</v>
       </c>
       <c r="E8" s="1"/>
-      <c r="I8" s="3" t="s">
+      <c r="I8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J8" s="3"/>
+      <c r="J8" s="2"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
@@ -669,7 +668,7 @@
       <c r="I9" t="s">
         <v>15</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9">
         <f>$H$1/0.012</f>
         <v>41.666666666666664</v>
       </c>
@@ -731,59 +730,247 @@
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-    </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B20" s="1"/>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" t="s">
+        <v>6</v>
+      </c>
+      <c r="D19" t="s">
+        <v>7</v>
+      </c>
+      <c r="G19" t="s">
+        <v>13</v>
+      </c>
+      <c r="H19" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="J19" t="s">
+        <v>5</v>
+      </c>
+      <c r="K19" t="s">
+        <v>6</v>
+      </c>
+      <c r="L19" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>0</v>
+      </c>
+      <c r="B20" s="1">
+        <v>0</v>
+      </c>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
-    </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
+      <c r="I20" t="s">
+        <v>14</v>
+      </c>
+      <c r="J20" s="1">
+        <f>$H$1/B28</f>
+        <v>2219.7558268590456</v>
+      </c>
+      <c r="K20">
+        <f t="shared" ref="K20" si="3">$H$1/C28</f>
+        <v>32.630685897017557</v>
+      </c>
+      <c r="L20">
+        <f t="shared" ref="L20" si="4">$H$1/D28</f>
+        <v>9302.325581395351</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>1</v>
+      </c>
+      <c r="B21" s="1">
+        <v>2.4999999999999999E-7</v>
+      </c>
+      <c r="C21" s="1">
+        <v>1.9999999999999999E-6</v>
+      </c>
+      <c r="D21" s="1">
+        <v>2.4999999999999999E-7</v>
+      </c>
       <c r="E21" s="1"/>
-    </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
+      <c r="I21" t="s">
+        <v>15</v>
+      </c>
+      <c r="J21">
+        <f>J20/24</f>
+        <v>92.489826119126903</v>
+      </c>
+      <c r="K21">
+        <f t="shared" ref="K21:L21" si="5">K20/24</f>
+        <v>1.3596119123757315</v>
+      </c>
+      <c r="L21">
+        <f t="shared" si="5"/>
+        <v>387.59689922480629</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>2</v>
+      </c>
+      <c r="B22" s="1">
+        <v>3.4999999999999997E-5</v>
+      </c>
+      <c r="C22" s="1">
+        <v>3.4999999999999997E-5</v>
+      </c>
+      <c r="D22" s="1">
+        <v>3.4999999999999997E-5</v>
+      </c>
       <c r="E22" s="1"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>3</v>
+      </c>
+      <c r="B23" s="1">
+        <v>1.2999999999999999E-5</v>
+      </c>
+      <c r="C23" s="1">
+        <v>2.5999999999999998E-5</v>
+      </c>
+      <c r="D23" s="1">
+        <v>3.0000000000000001E-6</v>
+      </c>
       <c r="E23" s="1"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B24" s="1">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="C24" s="1">
+        <v>1.6000000000000001E-4</v>
+      </c>
+      <c r="D24" s="1">
+        <v>1.0000000000000001E-5</v>
+      </c>
       <c r="E24" s="1"/>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
+      <c r="I24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="J24" s="2"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>9</v>
+      </c>
+      <c r="B25" s="1">
+        <v>1E-4</v>
+      </c>
+      <c r="C25" s="1">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="D25" s="1">
+        <v>5.0000000000000004E-6</v>
+      </c>
       <c r="E25" s="1"/>
+      <c r="I25" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J25" s="2"/>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>10</v>
+      </c>
+      <c r="B26" s="1">
+        <v>6.7000000000000002E-5</v>
+      </c>
+      <c r="C26" s="1">
+        <v>1E-4</v>
+      </c>
+      <c r="D26" s="1">
+        <v>4.9999999999999998E-7</v>
+      </c>
+      <c r="E26" s="1"/>
+      <c r="I26" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J26" s="2"/>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B27" t="s">
+        <v>5</v>
+      </c>
+      <c r="C27" t="s">
+        <v>6</v>
+      </c>
+      <c r="D27" t="s">
+        <v>7</v>
+      </c>
+      <c r="E27" s="1"/>
+      <c r="I27" t="s">
+        <v>15</v>
+      </c>
+      <c r="J27">
+        <f>$H$1/0.012</f>
+        <v>41.666666666666664</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>12</v>
+      </c>
+      <c r="B28" s="1">
+        <f>SUM(B20:B27)</f>
+        <v>2.2525E-4</v>
+      </c>
+      <c r="C28" s="1">
+        <f t="shared" ref="C28:D28" si="6">SUM(C20:C27)</f>
+        <v>1.5322999999999998E-2</v>
+      </c>
+      <c r="D28" s="1">
+        <f t="shared" si="6"/>
+        <v>5.3749999999999992E-5</v>
+      </c>
+      <c r="E28" s="1"/>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>11</v>
+      </c>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>